<commit_message>
corrected the column name in the excel sheet
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0DEF9D4-CBBD-5048-9C95-B1AF2C8D7004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB4B0CA-41D1-8449-B544-11EDC5AB0A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16100" xr2:uid="{205AF04C-A609-564D-A6E8-10952E504ABC}"/>
   </bookViews>
@@ -40,9 +40,6 @@
     <t>email</t>
   </si>
   <si>
-    <t>fullname</t>
-  </si>
-  <si>
     <t>nelsonterdoo1000@gmail.com</t>
   </si>
   <si>
@@ -59,6 +56,9 @@
   </si>
   <si>
     <t>Terdoo Nondo</t>
+  </si>
+  <si>
+    <t>full_name</t>
   </si>
 </sst>
 </file>
@@ -433,31 +433,31 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
         <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
         <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added more students for the demo
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Documents/python_scripts/college_election_portal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB4B0CA-41D1-8449-B544-11EDC5AB0A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCF764BC-84FA-F548-9EFE-402D6CB44D81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16100" xr2:uid="{205AF04C-A609-564D-A6E8-10952E504ABC}"/>
   </bookViews>
@@ -35,30 +35,156 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
   <si>
     <t>email</t>
   </si>
   <si>
-    <t>nelsonterdoo1000@gmail.com</t>
-  </si>
-  <si>
-    <t>Terdoo Nelson Nondo</t>
-  </si>
-  <si>
-    <t>nondo622@gmail.com</t>
-  </si>
-  <si>
-    <t>Nelson Terdoo</t>
-  </si>
-  <si>
-    <t>nelson@edufuntechnik.com</t>
-  </si>
-  <si>
-    <t>Terdoo Nondo</t>
-  </si>
-  <si>
     <t>full_name</t>
+  </si>
+  <si>
+    <t>victorjohnson537@gmail.com</t>
+  </si>
+  <si>
+    <t>harrychidiebere0013@gmail.com</t>
+  </si>
+  <si>
+    <t>Collinsezugwu74@gmail.com</t>
+  </si>
+  <si>
+    <t>emmanuelbonaventure8@gmail.com</t>
+  </si>
+  <si>
+    <t>faustinusikechukwu877@gmail.com</t>
+  </si>
+  <si>
+    <t>okolipeter587@gmail.com</t>
+  </si>
+  <si>
+    <t>ebubereine64@gmail.com</t>
+  </si>
+  <si>
+    <t>chukwuebukaofiaeli12@gmail.com</t>
+  </si>
+  <si>
+    <t>andrewnzeh16@gmail.com</t>
+  </si>
+  <si>
+    <t>salvagepascal6@gmail.com</t>
+  </si>
+  <si>
+    <t>Helenstudios001@email.com</t>
+  </si>
+  <si>
+    <t>chisomvitalis95@gmail.com</t>
+  </si>
+  <si>
+    <t>emmanuelobunike19@gmail.com</t>
+  </si>
+  <si>
+    <t>wattzchisom@gmail.com</t>
+  </si>
+  <si>
+    <t>oguguaesther584@gmail.com</t>
+  </si>
+  <si>
+    <t>simiigslaton@gmail.com</t>
+  </si>
+  <si>
+    <t>danielsomto420@gmail.com</t>
+  </si>
+  <si>
+    <t>odigweshedrach01@gmail.com</t>
+  </si>
+  <si>
+    <t>multiplejesus0808@gmail.com</t>
+  </si>
+  <si>
+    <t>mezemicheal386@gmail.com</t>
+  </si>
+  <si>
+    <t>peculiarozioma715@gmail.com</t>
+  </si>
+  <si>
+    <t>chiderachristian840@gmail.com</t>
+  </si>
+  <si>
+    <t>davidobinna924@gmail.com</t>
+  </si>
+  <si>
+    <t>Johnson Okechukwu Victor</t>
+  </si>
+  <si>
+    <t>OKOYE HARRISON CHIDIEBERE</t>
+  </si>
+  <si>
+    <t>Samuel Callmikelly Ezugwu</t>
+  </si>
+  <si>
+    <t>OKEKE EBUBECHUKWU BONAVENTURE EMMANUEL</t>
+  </si>
+  <si>
+    <t>Agbo ikechukwu faustinus</t>
+  </si>
+  <si>
+    <t>Okoli uchenna peter</t>
+  </si>
+  <si>
+    <t>Anamasonye Oluebube Miracle</t>
+  </si>
+  <si>
+    <t>OFIAELI CHUKWUEBUKA</t>
+  </si>
+  <si>
+    <t>Andy nzeh</t>
+  </si>
+  <si>
+    <t>Ezenwa Chinecherem Pascal</t>
+  </si>
+  <si>
+    <t>Helen</t>
+  </si>
+  <si>
+    <t>Ejike Vitalis chisom</t>
+  </si>
+  <si>
+    <t>Obunike Chukwuemerie Emmanuel</t>
+  </si>
+  <si>
+    <t>BONIFACE CHISOM EMMANUEL</t>
+  </si>
+  <si>
+    <t>Ogugua kosisochukwu Esther</t>
+  </si>
+  <si>
+    <t>Nwaogu Izuchukwu simon</t>
+  </si>
+  <si>
+    <t>Daniel Somto Okeke</t>
+  </si>
+  <si>
+    <t>Odigwe Chinemelum Shedrack</t>
+  </si>
+  <si>
+    <t>Amos Somto James</t>
+  </si>
+  <si>
+    <t>Meze michael</t>
+  </si>
+  <si>
+    <t>Ugwuja Peculiar Ozioma</t>
+  </si>
+  <si>
+    <t>Nwafor Christian Chidera</t>
+  </si>
+  <si>
+    <t>UDEGBUNAM OBINNA DAVID</t>
+  </si>
+  <si>
+    <t>Simeon James Chukwukaodinaka</t>
+  </si>
+  <si>
+    <t>jameschukwukaodinaka@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -74,12 +200,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Roboto"/>
     </font>
   </fonts>
   <fills count="2">
@@ -99,16 +222,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -421,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DB986F6-C945-824E-BAE1-932A8E371B3E}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.6640625" customWidth="1"/>
@@ -433,39 +554,210 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
         <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>4</v>
+      <c r="B3" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="B6" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>48</v>
+      </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{62D83B7E-7244-AD42-A5A3-E5777C23EEF9}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{8D4102E9-FD1B-CF42-A84E-1EB7D1C94EB3}"/>
-    <hyperlink ref="A4" r:id="rId3" xr:uid="{08E1B5B3-2DF6-D34B-B396-8CAB5892762B}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>